<commit_message>
added trainig and investment insights
</commit_message>
<xml_diff>
--- a/data/SDG_Goals_Targets_and_Indicators.xlsx
+++ b/data/SDG_Goals_Targets_and_Indicators.xlsx
@@ -5,22 +5,23 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ESGDATA.in\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ESGDATA.in\esgdata\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3412854-E435-43BC-AAED-6F22A1287D9C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46D91DA-A9A7-4B51-A489-AEC84880AEE0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>SDG</t>
   </si>
@@ -526,160 +527,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="125.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="125.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>17</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
         <v>18</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{800B2D08-A3B2-4A3A-9999-9AC674655E7E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>